<commit_message>
Actualizacion de formatos: Nuevas versiones detectadas
</commit_message>
<xml_diff>
--- a/Formatos/BITACORAS GFPI-F-147V4.xlsx
+++ b/Formatos/BITACORAS GFPI-F-147V4.xlsx
@@ -2704,408 +2704,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
@@ -3124,19 +2722,414 @@
         </ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="74" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDCFD71"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill>
@@ -3865,56 +3858,56 @@
       <c r="H2" s="7"/>
     </row>
     <row r="3" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="190" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="171"/>
-      <c r="D3" s="171"/>
-      <c r="E3" s="172"/>
+      <c r="C3" s="191"/>
+      <c r="D3" s="191"/>
+      <c r="E3" s="192"/>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="173" t="s">
+      <c r="B4" s="193" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="174"/>
-      <c r="D4" s="174"/>
-      <c r="E4" s="175"/>
+      <c r="C4" s="194"/>
+      <c r="D4" s="194"/>
+      <c r="E4" s="195"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="238" t="s">
+      <c r="B5" s="216" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="239"/>
-      <c r="D5" s="239"/>
-      <c r="E5" s="240"/>
+      <c r="C5" s="217"/>
+      <c r="D5" s="217"/>
+      <c r="E5" s="218"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
     </row>
     <row r="6" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="173" t="s">
+      <c r="B6" s="193" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="174"/>
-      <c r="D6" s="174"/>
-      <c r="E6" s="175"/>
+      <c r="C6" s="194"/>
+      <c r="D6" s="194"/>
+      <c r="E6" s="195"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
     </row>
     <row r="7" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="170" t="s">
+      <c r="B7" s="190" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="171"/>
-      <c r="D7" s="171"/>
-      <c r="E7" s="172"/>
+      <c r="C7" s="191"/>
+      <c r="D7" s="191"/>
+      <c r="E7" s="192"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
@@ -3926,45 +3919,45 @@
       <c r="C8" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="241" t="s">
+      <c r="D8" s="219" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="242"/>
+      <c r="E8" s="220"/>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="243" t="s">
+      <c r="B9" s="221" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="244"/>
-      <c r="D9" s="244"/>
-      <c r="E9" s="245"/>
+      <c r="C9" s="222"/>
+      <c r="D9" s="222"/>
+      <c r="E9" s="223"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
     </row>
     <row r="10" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="246" t="s">
+      <c r="B10" s="224" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="247"/>
-      <c r="D10" s="247"/>
-      <c r="E10" s="248"/>
+      <c r="C10" s="225"/>
+      <c r="D10" s="225"/>
+      <c r="E10" s="226"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="230" t="s">
+      <c r="B11" s="227" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="231"/>
-      <c r="D11" s="231"/>
-      <c r="E11" s="232"/>
+      <c r="C11" s="228"/>
+      <c r="D11" s="228"/>
+      <c r="E11" s="229"/>
     </row>
     <row r="12" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="221" t="s">
+      <c r="B12" s="212" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="222"/>
-      <c r="D12" s="223"/>
-      <c r="E12" s="224"/>
+      <c r="C12" s="213"/>
+      <c r="D12" s="214"/>
+      <c r="E12" s="215"/>
       <c r="F12" s="1"/>
       <c r="G12" s="34"/>
     </row>
@@ -3975,84 +3968,84 @@
       <c r="E13" s="75"/>
     </row>
     <row r="14" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="212" t="s">
+      <c r="B14" s="239" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="213"/>
-      <c r="D14" s="213"/>
-      <c r="E14" s="214"/>
+      <c r="C14" s="240"/>
+      <c r="D14" s="240"/>
+      <c r="E14" s="241"/>
     </row>
     <row r="15" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="215" t="s">
+      <c r="B15" s="242" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="216"/>
-      <c r="D15" s="216"/>
-      <c r="E15" s="217"/>
+      <c r="C15" s="243"/>
+      <c r="D15" s="243"/>
+      <c r="E15" s="244"/>
     </row>
     <row r="16" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="215" t="s">
+      <c r="B16" s="242" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="216"/>
-      <c r="D16" s="216"/>
-      <c r="E16" s="217"/>
+      <c r="C16" s="243"/>
+      <c r="D16" s="243"/>
+      <c r="E16" s="244"/>
     </row>
     <row r="17" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="225" t="s">
+      <c r="B17" s="248" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="226"/>
-      <c r="D17" s="226"/>
-      <c r="E17" s="227"/>
+      <c r="C17" s="249"/>
+      <c r="D17" s="249"/>
+      <c r="E17" s="250"/>
     </row>
     <row r="18" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="215" t="s">
+      <c r="B18" s="242" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="216"/>
-      <c r="D18" s="216"/>
-      <c r="E18" s="217"/>
+      <c r="C18" s="243"/>
+      <c r="D18" s="243"/>
+      <c r="E18" s="244"/>
     </row>
     <row r="19" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="215" t="s">
+      <c r="B19" s="242" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="216"/>
-      <c r="D19" s="216"/>
-      <c r="E19" s="217"/>
+      <c r="C19" s="243"/>
+      <c r="D19" s="243"/>
+      <c r="E19" s="244"/>
     </row>
     <row r="20" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="218" t="s">
+      <c r="B20" s="245" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="219"/>
-      <c r="D20" s="219"/>
-      <c r="E20" s="220"/>
+      <c r="C20" s="246"/>
+      <c r="D20" s="246"/>
+      <c r="E20" s="247"/>
     </row>
     <row r="21" spans="2:6" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="221" t="s">
+      <c r="B21" s="212" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="222"/>
-      <c r="D21" s="223"/>
-      <c r="E21" s="224"/>
+      <c r="C21" s="213"/>
+      <c r="D21" s="214"/>
+      <c r="E21" s="215"/>
     </row>
     <row r="22" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="230" t="s">
+      <c r="B22" s="227" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="231"/>
-      <c r="D22" s="231" t="s">
+      <c r="C22" s="228"/>
+      <c r="D22" s="228" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="232"/>
+      <c r="E22" s="229"/>
     </row>
     <row r="23" spans="2:6" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="233"/>
-      <c r="C23" s="234"/>
-      <c r="D23" s="234"/>
-      <c r="E23" s="235"/>
+      <c r="B23" s="230"/>
+      <c r="C23" s="231"/>
+      <c r="D23" s="231"/>
+      <c r="E23" s="232"/>
     </row>
     <row r="24" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="68" t="s">
@@ -4061,10 +4054,10 @@
       <c r="C24" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="236" t="s">
+      <c r="D24" s="233" t="s">
         <v>25</v>
       </c>
-      <c r="E24" s="237"/>
+      <c r="E24" s="234"/>
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -4074,8 +4067,8 @@
       <c r="C25" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="D25" s="228"/>
-      <c r="E25" s="229"/>
+      <c r="D25" s="235"/>
+      <c r="E25" s="236"/>
     </row>
     <row r="26" spans="2:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B26" s="57" t="s">
@@ -4084,8 +4077,8 @@
       <c r="C26" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="228"/>
-      <c r="E26" s="229"/>
+      <c r="D26" s="235"/>
+      <c r="E26" s="236"/>
     </row>
     <row r="27" spans="2:6" ht="45" x14ac:dyDescent="0.25">
       <c r="B27" s="59" t="s">
@@ -4094,8 +4087,8 @@
       <c r="C27" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="D27" s="228"/>
-      <c r="E27" s="229"/>
+      <c r="D27" s="235"/>
+      <c r="E27" s="236"/>
     </row>
     <row r="28" spans="2:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="69" t="s">
@@ -4104,8 +4097,8 @@
       <c r="C28" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="D28" s="228"/>
-      <c r="E28" s="229"/>
+      <c r="D28" s="235"/>
+      <c r="E28" s="236"/>
     </row>
     <row r="29" spans="2:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="69" t="s">
@@ -4114,10 +4107,10 @@
       <c r="C29" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="D29" s="228" t="s">
+      <c r="D29" s="235" t="s">
         <v>36</v>
       </c>
-      <c r="E29" s="229" t="s">
+      <c r="E29" s="236" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4128,10 +4121,10 @@
       <c r="C30" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="228" t="s">
+      <c r="D30" s="235" t="s">
         <v>39</v>
       </c>
-      <c r="E30" s="229" t="s">
+      <c r="E30" s="236" t="s">
         <v>39</v>
       </c>
     </row>
@@ -4142,8 +4135,8 @@
       <c r="C31" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="228"/>
-      <c r="E31" s="229"/>
+      <c r="D31" s="235"/>
+      <c r="E31" s="236"/>
     </row>
     <row r="32" spans="2:6" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="69" t="s">
@@ -4152,10 +4145,10 @@
       <c r="C32" s="56" t="s">
         <v>43</v>
       </c>
-      <c r="D32" s="228" t="s">
+      <c r="D32" s="235" t="s">
         <v>44</v>
       </c>
-      <c r="E32" s="229" t="s">
+      <c r="E32" s="236" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4166,8 +4159,8 @@
       <c r="C33" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="D33" s="228"/>
-      <c r="E33" s="229"/>
+      <c r="D33" s="235"/>
+      <c r="E33" s="236"/>
     </row>
     <row r="34" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B34" s="69" t="s">
@@ -4176,8 +4169,8 @@
       <c r="C34" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="D34" s="228"/>
-      <c r="E34" s="229"/>
+      <c r="D34" s="235"/>
+      <c r="E34" s="236"/>
     </row>
     <row r="35" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B35" s="69" t="s">
@@ -4186,8 +4179,8 @@
       <c r="C35" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="D35" s="228"/>
-      <c r="E35" s="229"/>
+      <c r="D35" s="235"/>
+      <c r="E35" s="236"/>
     </row>
     <row r="36" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B36" s="69" t="s">
@@ -4196,8 +4189,8 @@
       <c r="C36" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="D36" s="228"/>
-      <c r="E36" s="229"/>
+      <c r="D36" s="235"/>
+      <c r="E36" s="236"/>
     </row>
     <row r="37" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B37" s="69" t="s">
@@ -4206,8 +4199,8 @@
       <c r="C37" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="D37" s="228"/>
-      <c r="E37" s="229"/>
+      <c r="D37" s="235"/>
+      <c r="E37" s="236"/>
     </row>
     <row r="38" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B38" s="69" t="s">
@@ -4216,8 +4209,8 @@
       <c r="C38" s="56" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="228"/>
-      <c r="E38" s="229"/>
+      <c r="D38" s="235"/>
+      <c r="E38" s="236"/>
     </row>
     <row r="39" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B39" s="69" t="s">
@@ -4226,8 +4219,8 @@
       <c r="C39" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="D39" s="228"/>
-      <c r="E39" s="229"/>
+      <c r="D39" s="235"/>
+      <c r="E39" s="236"/>
     </row>
     <row r="40" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B40" s="69" t="s">
@@ -4236,8 +4229,8 @@
       <c r="C40" s="56" t="s">
         <v>59</v>
       </c>
-      <c r="D40" s="228"/>
-      <c r="E40" s="229"/>
+      <c r="D40" s="235"/>
+      <c r="E40" s="236"/>
     </row>
     <row r="41" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B41" s="69" t="s">
@@ -4246,8 +4239,8 @@
       <c r="C41" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="D41" s="228"/>
-      <c r="E41" s="229"/>
+      <c r="D41" s="235"/>
+      <c r="E41" s="236"/>
     </row>
     <row r="42" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B42" s="69" t="s">
@@ -4256,8 +4249,8 @@
       <c r="C42" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="D42" s="228"/>
-      <c r="E42" s="229"/>
+      <c r="D42" s="235"/>
+      <c r="E42" s="236"/>
     </row>
     <row r="43" spans="2:5" ht="409.5" x14ac:dyDescent="0.25">
       <c r="B43" s="69" t="s">
@@ -4266,10 +4259,10 @@
       <c r="C43" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="D43" s="228" t="s">
+      <c r="D43" s="235" t="s">
         <v>65</v>
       </c>
-      <c r="E43" s="229" t="s">
+      <c r="E43" s="236" t="s">
         <v>65</v>
       </c>
     </row>
@@ -4280,8 +4273,8 @@
       <c r="C44" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="228"/>
-      <c r="E44" s="229"/>
+      <c r="D44" s="235"/>
+      <c r="E44" s="236"/>
     </row>
     <row r="45" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B45" s="69" t="s">
@@ -4290,8 +4283,8 @@
       <c r="C45" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="D45" s="228"/>
-      <c r="E45" s="229"/>
+      <c r="D45" s="235"/>
+      <c r="E45" s="236"/>
     </row>
     <row r="46" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B46" s="69" t="s">
@@ -4300,8 +4293,8 @@
       <c r="C46" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="D46" s="228"/>
-      <c r="E46" s="229"/>
+      <c r="D46" s="235"/>
+      <c r="E46" s="236"/>
     </row>
     <row r="47" spans="2:5" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="69" t="s">
@@ -4310,10 +4303,10 @@
       <c r="C47" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="D47" s="228" t="s">
+      <c r="D47" s="235" t="s">
         <v>74</v>
       </c>
-      <c r="E47" s="229" t="s">
+      <c r="E47" s="236" t="s">
         <v>74</v>
       </c>
     </row>
@@ -4324,8 +4317,8 @@
       <c r="C48" s="56" t="s">
         <v>76</v>
       </c>
-      <c r="D48" s="228"/>
-      <c r="E48" s="229"/>
+      <c r="D48" s="235"/>
+      <c r="E48" s="236"/>
     </row>
     <row r="49" spans="2:5" ht="146.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="69" t="s">
@@ -4334,10 +4327,10 @@
       <c r="C49" s="56" t="s">
         <v>78</v>
       </c>
-      <c r="D49" s="228" t="s">
+      <c r="D49" s="235" t="s">
         <v>79</v>
       </c>
-      <c r="E49" s="229" t="s">
+      <c r="E49" s="236" t="s">
         <v>79</v>
       </c>
     </row>
@@ -4348,10 +4341,10 @@
       <c r="C50" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="D50" s="228" t="s">
+      <c r="D50" s="235" t="s">
         <v>82</v>
       </c>
-      <c r="E50" s="229" t="s">
+      <c r="E50" s="236" t="s">
         <v>83</v>
       </c>
     </row>
@@ -4362,10 +4355,10 @@
       <c r="C51" s="61" t="s">
         <v>85</v>
       </c>
-      <c r="D51" s="228" t="s">
+      <c r="D51" s="235" t="s">
         <v>86</v>
       </c>
-      <c r="E51" s="229" t="s">
+      <c r="E51" s="236" t="s">
         <v>86</v>
       </c>
     </row>
@@ -4376,8 +4369,8 @@
       <c r="C52" s="56" t="s">
         <v>88</v>
       </c>
-      <c r="D52" s="228"/>
-      <c r="E52" s="229"/>
+      <c r="D52" s="235"/>
+      <c r="E52" s="236"/>
     </row>
     <row r="53" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B53" s="69" t="s">
@@ -4386,8 +4379,8 @@
       <c r="C53" s="61" t="s">
         <v>90</v>
       </c>
-      <c r="D53" s="228"/>
-      <c r="E53" s="229"/>
+      <c r="D53" s="235"/>
+      <c r="E53" s="236"/>
     </row>
     <row r="54" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B54" s="69" t="s">
@@ -4396,8 +4389,8 @@
       <c r="C54" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="D54" s="228"/>
-      <c r="E54" s="229"/>
+      <c r="D54" s="235"/>
+      <c r="E54" s="236"/>
     </row>
     <row r="55" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B55" s="69" t="s">
@@ -4406,8 +4399,8 @@
       <c r="C55" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D55" s="228"/>
-      <c r="E55" s="229"/>
+      <c r="D55" s="235"/>
+      <c r="E55" s="236"/>
     </row>
     <row r="56" spans="2:5" ht="75" x14ac:dyDescent="0.25">
       <c r="B56" s="70" t="s">
@@ -4416,8 +4409,8 @@
       <c r="C56" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D56" s="228"/>
-      <c r="E56" s="229"/>
+      <c r="D56" s="235"/>
+      <c r="E56" s="236"/>
     </row>
     <row r="57" spans="2:5" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B57" s="71" t="s">
@@ -4426,10 +4419,10 @@
       <c r="C57" s="72" t="s">
         <v>97</v>
       </c>
-      <c r="D57" s="210" t="s">
+      <c r="D57" s="237" t="s">
         <v>98</v>
       </c>
-      <c r="E57" s="211" t="s">
+      <c r="E57" s="238" t="s">
         <v>98</v>
       </c>
     </row>
@@ -4447,44 +4440,6 @@
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
     <mergeCell ref="D57:E57"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B19:E19"/>
@@ -4501,6 +4456,44 @@
     <mergeCell ref="D56:E56"/>
     <mergeCell ref="D47:E47"/>
     <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="B11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4590,14 +4583,14 @@
       <c r="Z2" s="9"/>
     </row>
     <row r="3" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="170" t="s">
+      <c r="B3" s="190" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="171"/>
-      <c r="D3" s="171"/>
-      <c r="E3" s="171"/>
-      <c r="F3" s="171"/>
-      <c r="G3" s="172"/>
+      <c r="C3" s="191"/>
+      <c r="D3" s="191"/>
+      <c r="E3" s="191"/>
+      <c r="F3" s="191"/>
+      <c r="G3" s="192"/>
       <c r="H3" s="10"/>
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
@@ -4619,14 +4612,14 @@
       <c r="Z3" s="9"/>
     </row>
     <row r="4" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="173" t="s">
+      <c r="B4" s="193" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="174"/>
-      <c r="D4" s="174"/>
-      <c r="E4" s="174"/>
-      <c r="F4" s="174"/>
-      <c r="G4" s="175"/>
+      <c r="C4" s="194"/>
+      <c r="D4" s="194"/>
+      <c r="E4" s="194"/>
+      <c r="F4" s="194"/>
+      <c r="G4" s="195"/>
       <c r="H4" s="10"/>
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
@@ -4648,14 +4641,14 @@
       <c r="Z4" s="9"/>
     </row>
     <row r="5" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="170" t="s">
+      <c r="B5" s="190" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="171"/>
-      <c r="D5" s="171"/>
-      <c r="E5" s="171"/>
-      <c r="F5" s="171"/>
-      <c r="G5" s="172"/>
+      <c r="C5" s="191"/>
+      <c r="D5" s="191"/>
+      <c r="E5" s="191"/>
+      <c r="F5" s="191"/>
+      <c r="G5" s="192"/>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
       <c r="J5" s="9"/>
@@ -4677,14 +4670,14 @@
       <c r="Z5" s="9"/>
     </row>
     <row r="6" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="173" t="s">
+      <c r="B6" s="193" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="174"/>
-      <c r="D6" s="174"/>
-      <c r="E6" s="174"/>
-      <c r="F6" s="174"/>
-      <c r="G6" s="175"/>
+      <c r="C6" s="194"/>
+      <c r="D6" s="194"/>
+      <c r="E6" s="194"/>
+      <c r="F6" s="194"/>
+      <c r="G6" s="195"/>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
       <c r="J6" s="9"/>
@@ -4706,14 +4699,14 @@
       <c r="Z6" s="9"/>
     </row>
     <row r="7" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="170" t="s">
+      <c r="B7" s="190" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="171"/>
-      <c r="D7" s="171"/>
-      <c r="E7" s="171"/>
-      <c r="F7" s="171"/>
-      <c r="G7" s="172"/>
+      <c r="C7" s="191"/>
+      <c r="D7" s="191"/>
+      <c r="E7" s="191"/>
+      <c r="F7" s="191"/>
+      <c r="G7" s="192"/>
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
@@ -4738,19 +4731,19 @@
       <c r="B8" s="133" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="283" t="b">
+      <c r="C8" s="158" t="b">
         <v>0</v>
       </c>
       <c r="D8" s="134" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="283" t="b">
+      <c r="E8" s="158" t="b">
         <v>0</v>
       </c>
       <c r="F8" s="134" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="284" t="b">
+      <c r="G8" s="159" t="b">
         <v>0</v>
       </c>
       <c r="H8" s="9"/>
@@ -4903,12 +4896,12 @@
       <c r="Y13" s="18"/>
     </row>
     <row r="14" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="161"/>
-      <c r="C14" s="163"/>
-      <c r="D14" s="162"/>
-      <c r="E14" s="158"/>
-      <c r="F14" s="159"/>
-      <c r="G14" s="160"/>
+      <c r="B14" s="160"/>
+      <c r="C14" s="161"/>
+      <c r="D14" s="198"/>
+      <c r="E14" s="207"/>
+      <c r="F14" s="208"/>
+      <c r="G14" s="209"/>
       <c r="H14" s="20"/>
       <c r="I14" s="20"/>
       <c r="J14" s="20"/>
@@ -4980,12 +4973,12 @@
       <c r="Z16" s="12"/>
     </row>
     <row r="17" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="161"/>
-      <c r="C17" s="162"/>
+      <c r="B17" s="160"/>
+      <c r="C17" s="198"/>
       <c r="D17" s="142"/>
       <c r="E17" s="143"/>
-      <c r="F17" s="176"/>
-      <c r="G17" s="177"/>
+      <c r="F17" s="196"/>
+      <c r="G17" s="197"/>
       <c r="H17" s="20"/>
       <c r="I17" s="20"/>
       <c r="K17" s="20"/>
@@ -5053,12 +5046,12 @@
       <c r="Z19" s="12"/>
     </row>
     <row r="20" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="161"/>
-      <c r="C20" s="162"/>
+      <c r="B20" s="160"/>
+      <c r="C20" s="198"/>
       <c r="D20" s="141"/>
       <c r="E20" s="144"/>
-      <c r="F20" s="178"/>
-      <c r="G20" s="179"/>
+      <c r="F20" s="199"/>
+      <c r="G20" s="162"/>
       <c r="H20" s="20"/>
       <c r="L20" s="20"/>
       <c r="M20" s="20"/>
@@ -5100,14 +5093,14 @@
       <c r="Y21" s="15"/>
     </row>
     <row r="22" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="184" t="s">
+      <c r="B22" s="204" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="185"/>
-      <c r="D22" s="185"/>
-      <c r="E22" s="185"/>
-      <c r="F22" s="185"/>
-      <c r="G22" s="186"/>
+      <c r="C22" s="205"/>
+      <c r="D22" s="205"/>
+      <c r="E22" s="205"/>
+      <c r="F22" s="205"/>
+      <c r="G22" s="206"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="9"/>
@@ -5132,13 +5125,13 @@
       <c r="B23" s="131" t="s">
         <v>106</v>
       </c>
-      <c r="C23" s="180"/>
-      <c r="D23" s="181"/>
+      <c r="C23" s="200"/>
+      <c r="D23" s="201"/>
       <c r="E23" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="F23" s="182"/>
-      <c r="G23" s="183"/>
+      <c r="F23" s="202"/>
+      <c r="G23" s="203"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
       <c r="J23" s="9"/>
@@ -5282,10 +5275,10 @@
       </c>
       <c r="D28" s="146"/>
       <c r="E28" s="46"/>
-      <c r="F28" s="164" t="s">
+      <c r="F28" s="210" t="s">
         <v>114</v>
       </c>
-      <c r="G28" s="165"/>
+      <c r="G28" s="211"/>
       <c r="H28" s="18"/>
       <c r="I28" s="18"/>
       <c r="J28" s="20"/>
@@ -5312,8 +5305,8 @@
       <c r="E29" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="F29" s="164"/>
-      <c r="G29" s="165"/>
+      <c r="F29" s="210"/>
+      <c r="G29" s="211"/>
       <c r="H29" s="18"/>
       <c r="I29" s="18"/>
       <c r="J29" s="20"/>
@@ -5649,12 +5642,12 @@
       <c r="Y39" s="18"/>
     </row>
     <row r="40" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="187"/>
-      <c r="C40" s="188"/>
-      <c r="D40" s="191"/>
-      <c r="E40" s="191"/>
-      <c r="F40" s="191"/>
-      <c r="G40" s="193"/>
+      <c r="B40" s="178"/>
+      <c r="C40" s="179"/>
+      <c r="D40" s="182"/>
+      <c r="E40" s="182"/>
+      <c r="F40" s="182"/>
+      <c r="G40" s="184"/>
       <c r="H40" s="20"/>
       <c r="I40" s="18"/>
       <c r="J40" s="18"/>
@@ -5675,12 +5668,12 @@
       <c r="Y40" s="18"/>
     </row>
     <row r="41" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="189"/>
-      <c r="C41" s="190"/>
-      <c r="D41" s="192"/>
-      <c r="E41" s="192"/>
-      <c r="F41" s="192"/>
-      <c r="G41" s="194"/>
+      <c r="B41" s="180"/>
+      <c r="C41" s="181"/>
+      <c r="D41" s="183"/>
+      <c r="E41" s="183"/>
+      <c r="F41" s="183"/>
+      <c r="G41" s="185"/>
       <c r="H41" s="20"/>
       <c r="I41" s="18"/>
       <c r="J41" s="18"/>
@@ -5701,12 +5694,12 @@
       <c r="Y41" s="18"/>
     </row>
     <row r="42" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="187"/>
-      <c r="C42" s="188"/>
-      <c r="D42" s="191"/>
-      <c r="E42" s="191"/>
-      <c r="F42" s="191"/>
-      <c r="G42" s="193"/>
+      <c r="B42" s="178"/>
+      <c r="C42" s="179"/>
+      <c r="D42" s="182"/>
+      <c r="E42" s="182"/>
+      <c r="F42" s="182"/>
+      <c r="G42" s="184"/>
       <c r="H42" s="20"/>
       <c r="I42" s="18"/>
       <c r="J42" s="18"/>
@@ -5727,12 +5720,12 @@
       <c r="Y42" s="18"/>
     </row>
     <row r="43" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="189"/>
-      <c r="C43" s="190"/>
-      <c r="D43" s="192"/>
-      <c r="E43" s="192"/>
-      <c r="F43" s="192"/>
-      <c r="G43" s="194"/>
+      <c r="B43" s="180"/>
+      <c r="C43" s="181"/>
+      <c r="D43" s="183"/>
+      <c r="E43" s="183"/>
+      <c r="F43" s="183"/>
+      <c r="G43" s="185"/>
       <c r="H43" s="20"/>
       <c r="I43" s="18"/>
       <c r="J43" s="18"/>
@@ -5753,12 +5746,12 @@
       <c r="Y43" s="18"/>
     </row>
     <row r="44" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="187"/>
-      <c r="C44" s="188"/>
-      <c r="D44" s="191"/>
-      <c r="E44" s="191"/>
-      <c r="F44" s="191"/>
-      <c r="G44" s="193"/>
+      <c r="B44" s="178"/>
+      <c r="C44" s="179"/>
+      <c r="D44" s="182"/>
+      <c r="E44" s="182"/>
+      <c r="F44" s="182"/>
+      <c r="G44" s="184"/>
       <c r="H44" s="20"/>
       <c r="I44" s="18"/>
       <c r="J44" s="18"/>
@@ -5779,12 +5772,12 @@
       <c r="Y44" s="18"/>
     </row>
     <row r="45" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="189"/>
-      <c r="C45" s="190"/>
-      <c r="D45" s="192"/>
-      <c r="E45" s="192"/>
-      <c r="F45" s="192"/>
-      <c r="G45" s="194"/>
+      <c r="B45" s="180"/>
+      <c r="C45" s="181"/>
+      <c r="D45" s="183"/>
+      <c r="E45" s="183"/>
+      <c r="F45" s="183"/>
+      <c r="G45" s="185"/>
       <c r="H45" s="20"/>
       <c r="I45" s="18"/>
       <c r="J45" s="18"/>
@@ -5805,12 +5798,12 @@
       <c r="Y45" s="18"/>
     </row>
     <row r="46" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="187"/>
-      <c r="C46" s="188"/>
-      <c r="D46" s="191"/>
-      <c r="E46" s="191"/>
-      <c r="F46" s="191"/>
-      <c r="G46" s="193"/>
+      <c r="B46" s="178"/>
+      <c r="C46" s="179"/>
+      <c r="D46" s="182"/>
+      <c r="E46" s="182"/>
+      <c r="F46" s="182"/>
+      <c r="G46" s="184"/>
       <c r="H46" s="20"/>
       <c r="I46" s="18"/>
       <c r="J46" s="18"/>
@@ -5831,12 +5824,12 @@
       <c r="Y46" s="18"/>
     </row>
     <row r="47" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="189"/>
-      <c r="C47" s="190"/>
-      <c r="D47" s="192"/>
-      <c r="E47" s="192"/>
-      <c r="F47" s="192"/>
-      <c r="G47" s="194"/>
+      <c r="B47" s="180"/>
+      <c r="C47" s="181"/>
+      <c r="D47" s="183"/>
+      <c r="E47" s="183"/>
+      <c r="F47" s="183"/>
+      <c r="G47" s="185"/>
       <c r="H47" s="20"/>
       <c r="I47" s="18"/>
       <c r="J47" s="18"/>
@@ -5857,12 +5850,12 @@
       <c r="Y47" s="18"/>
     </row>
     <row r="48" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="187"/>
-      <c r="C48" s="188"/>
-      <c r="D48" s="191"/>
-      <c r="E48" s="191"/>
-      <c r="F48" s="191"/>
-      <c r="G48" s="193"/>
+      <c r="B48" s="178"/>
+      <c r="C48" s="179"/>
+      <c r="D48" s="182"/>
+      <c r="E48" s="182"/>
+      <c r="F48" s="182"/>
+      <c r="G48" s="184"/>
       <c r="H48" s="20"/>
       <c r="I48" s="18"/>
       <c r="J48" s="18"/>
@@ -5883,12 +5876,12 @@
       <c r="Y48" s="18"/>
     </row>
     <row r="49" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="189"/>
-      <c r="C49" s="190"/>
-      <c r="D49" s="192"/>
-      <c r="E49" s="192"/>
-      <c r="F49" s="192"/>
-      <c r="G49" s="194"/>
+      <c r="B49" s="180"/>
+      <c r="C49" s="181"/>
+      <c r="D49" s="183"/>
+      <c r="E49" s="183"/>
+      <c r="F49" s="183"/>
+      <c r="G49" s="185"/>
       <c r="H49" s="20"/>
       <c r="I49" s="18"/>
       <c r="J49" s="18"/>
@@ -5909,12 +5902,12 @@
       <c r="Y49" s="18"/>
     </row>
     <row r="50" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="187"/>
-      <c r="C50" s="188"/>
-      <c r="D50" s="191"/>
-      <c r="E50" s="191"/>
-      <c r="F50" s="191"/>
-      <c r="G50" s="193"/>
+      <c r="B50" s="178"/>
+      <c r="C50" s="179"/>
+      <c r="D50" s="182"/>
+      <c r="E50" s="182"/>
+      <c r="F50" s="182"/>
+      <c r="G50" s="184"/>
       <c r="H50" s="20"/>
       <c r="I50" s="18"/>
       <c r="J50" s="18"/>
@@ -5935,12 +5928,12 @@
       <c r="Y50" s="18"/>
     </row>
     <row r="51" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="189"/>
-      <c r="C51" s="190"/>
-      <c r="D51" s="192"/>
-      <c r="E51" s="192"/>
-      <c r="F51" s="192"/>
-      <c r="G51" s="194"/>
+      <c r="B51" s="180"/>
+      <c r="C51" s="181"/>
+      <c r="D51" s="183"/>
+      <c r="E51" s="183"/>
+      <c r="F51" s="183"/>
+      <c r="G51" s="185"/>
       <c r="H51" s="20"/>
       <c r="I51" s="18"/>
       <c r="J51" s="18"/>
@@ -5961,12 +5954,12 @@
       <c r="Y51" s="18"/>
     </row>
     <row r="52" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="187"/>
-      <c r="C52" s="188"/>
-      <c r="D52" s="191"/>
-      <c r="E52" s="191"/>
-      <c r="F52" s="191"/>
-      <c r="G52" s="193"/>
+      <c r="B52" s="178"/>
+      <c r="C52" s="179"/>
+      <c r="D52" s="182"/>
+      <c r="E52" s="182"/>
+      <c r="F52" s="182"/>
+      <c r="G52" s="184"/>
       <c r="H52" s="20"/>
       <c r="I52" s="18"/>
       <c r="J52" s="18"/>
@@ -5987,12 +5980,12 @@
       <c r="Y52" s="18"/>
     </row>
     <row r="53" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="189"/>
-      <c r="C53" s="190"/>
-      <c r="D53" s="192"/>
-      <c r="E53" s="192"/>
-      <c r="F53" s="192"/>
-      <c r="G53" s="194"/>
+      <c r="B53" s="180"/>
+      <c r="C53" s="181"/>
+      <c r="D53" s="183"/>
+      <c r="E53" s="183"/>
+      <c r="F53" s="183"/>
+      <c r="G53" s="185"/>
       <c r="H53" s="20"/>
       <c r="I53" s="18"/>
       <c r="J53" s="18"/>
@@ -6067,14 +6060,14 @@
       <c r="Y55" s="22"/>
     </row>
     <row r="56" spans="2:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="167" t="s">
+      <c r="B56" s="187" t="s">
         <v>147</v>
       </c>
-      <c r="C56" s="168"/>
-      <c r="D56" s="168"/>
-      <c r="E56" s="168"/>
-      <c r="F56" s="168"/>
-      <c r="G56" s="169"/>
+      <c r="C56" s="188"/>
+      <c r="D56" s="188"/>
+      <c r="E56" s="188"/>
+      <c r="F56" s="188"/>
+      <c r="G56" s="189"/>
       <c r="H56" s="22"/>
       <c r="I56" s="22"/>
       <c r="J56" s="22"/>
@@ -6216,11 +6209,11 @@
       <c r="D61" s="104" t="s">
         <v>84</v>
       </c>
-      <c r="E61" s="195"/>
+      <c r="E61" s="163"/>
       <c r="F61" s="104" t="s">
         <v>152</v>
       </c>
-      <c r="G61" s="195"/>
+      <c r="G61" s="163"/>
       <c r="H61" s="18"/>
       <c r="I61" s="18"/>
       <c r="J61" s="18"/>
@@ -6245,9 +6238,9 @@
       <c r="B62" s="155"/>
       <c r="C62" s="156"/>
       <c r="D62" s="101"/>
-      <c r="E62" s="196"/>
+      <c r="E62" s="164"/>
       <c r="F62" s="101"/>
-      <c r="G62" s="196"/>
+      <c r="G62" s="164"/>
       <c r="H62" s="18"/>
       <c r="I62" s="18"/>
       <c r="J62" s="18"/>
@@ -6324,9 +6317,9 @@
       <c r="Z64" s="18"/>
     </row>
     <row r="65" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="197"/>
-      <c r="C65" s="197"/>
-      <c r="D65" s="197"/>
+      <c r="B65" s="165"/>
+      <c r="C65" s="165"/>
+      <c r="D65" s="165"/>
       <c r="E65" s="17"/>
       <c r="F65" s="17"/>
       <c r="G65" s="17"/>
@@ -6351,9 +6344,9 @@
       <c r="Z65" s="18"/>
     </row>
     <row r="66" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="197"/>
-      <c r="C66" s="197"/>
-      <c r="D66" s="197"/>
+      <c r="B66" s="165"/>
+      <c r="C66" s="165"/>
+      <c r="D66" s="165"/>
       <c r="E66" s="17"/>
       <c r="F66" s="17"/>
       <c r="G66" s="17"/>
@@ -6378,9 +6371,9 @@
       <c r="Z66" s="18"/>
     </row>
     <row r="67" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="198"/>
-      <c r="C67" s="198"/>
-      <c r="D67" s="198"/>
+      <c r="B67" s="166"/>
+      <c r="C67" s="166"/>
+      <c r="D67" s="166"/>
       <c r="F67" s="157"/>
       <c r="G67" s="18"/>
       <c r="H67" s="18"/>
@@ -6404,11 +6397,11 @@
       <c r="Z67" s="18"/>
     </row>
     <row r="68" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="166" t="s">
+      <c r="B68" s="186" t="s">
         <v>89</v>
       </c>
-      <c r="C68" s="166"/>
-      <c r="D68" s="166"/>
+      <c r="C68" s="186"/>
+      <c r="D68" s="186"/>
       <c r="F68" s="19" t="s">
         <v>91</v>
       </c>
@@ -6434,11 +6427,11 @@
       <c r="Z68" s="18"/>
     </row>
     <row r="69" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B69" s="199"/>
-      <c r="C69" s="199"/>
-      <c r="D69" s="199"/>
-      <c r="F69" s="202"/>
-      <c r="G69" s="202"/>
+      <c r="B69" s="167"/>
+      <c r="C69" s="167"/>
+      <c r="D69" s="167"/>
+      <c r="F69" s="170"/>
+      <c r="G69" s="170"/>
       <c r="H69" s="18"/>
       <c r="I69" s="18"/>
       <c r="J69" s="18"/>
@@ -6460,11 +6453,11 @@
       <c r="Z69" s="18"/>
     </row>
     <row r="70" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B70" s="199"/>
-      <c r="C70" s="199"/>
-      <c r="D70" s="199"/>
-      <c r="F70" s="202"/>
-      <c r="G70" s="202"/>
+      <c r="B70" s="167"/>
+      <c r="C70" s="167"/>
+      <c r="D70" s="167"/>
+      <c r="F70" s="170"/>
+      <c r="G70" s="170"/>
       <c r="H70" s="18"/>
       <c r="I70" s="18"/>
       <c r="J70" s="18"/>
@@ -6486,11 +6479,11 @@
       <c r="Z70" s="18"/>
     </row>
     <row r="71" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="200"/>
-      <c r="C71" s="200"/>
-      <c r="D71" s="200"/>
-      <c r="F71" s="203"/>
-      <c r="G71" s="203"/>
+      <c r="B71" s="168"/>
+      <c r="C71" s="168"/>
+      <c r="D71" s="168"/>
+      <c r="F71" s="171"/>
+      <c r="G71" s="171"/>
       <c r="H71" s="18"/>
       <c r="I71" s="18"/>
       <c r="J71" s="18"/>
@@ -6512,15 +6505,15 @@
       <c r="Z71" s="18"/>
     </row>
     <row r="72" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B72" s="201" t="s">
+      <c r="B72" s="169" t="s">
         <v>93</v>
       </c>
-      <c r="C72" s="201"/>
-      <c r="D72" s="201"/>
-      <c r="F72" s="166" t="s">
+      <c r="C72" s="169"/>
+      <c r="D72" s="169"/>
+      <c r="F72" s="186" t="s">
         <v>154</v>
       </c>
-      <c r="G72" s="166"/>
+      <c r="G72" s="186"/>
       <c r="H72" s="18"/>
       <c r="I72" s="18"/>
       <c r="J72" s="18"/>
@@ -6598,14 +6591,14 @@
       <c r="Z74" s="18"/>
     </row>
     <row r="75" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="204" t="s">
+      <c r="B75" s="172" t="s">
         <v>156</v>
       </c>
-      <c r="C75" s="205"/>
-      <c r="D75" s="205"/>
-      <c r="E75" s="205"/>
-      <c r="F75" s="205"/>
-      <c r="G75" s="206"/>
+      <c r="C75" s="173"/>
+      <c r="D75" s="173"/>
+      <c r="E75" s="173"/>
+      <c r="F75" s="173"/>
+      <c r="G75" s="174"/>
       <c r="H75" s="10"/>
       <c r="I75" s="9"/>
       <c r="J75" s="9"/>
@@ -6627,14 +6620,14 @@
       <c r="Z75" s="9"/>
     </row>
     <row r="76" spans="2:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="207" t="s">
+      <c r="B76" s="175" t="s">
         <v>157</v>
       </c>
-      <c r="C76" s="208"/>
-      <c r="D76" s="208"/>
-      <c r="E76" s="208"/>
-      <c r="F76" s="208"/>
-      <c r="G76" s="209"/>
+      <c r="C76" s="176"/>
+      <c r="D76" s="176"/>
+      <c r="E76" s="176"/>
+      <c r="F76" s="176"/>
+      <c r="G76" s="177"/>
       <c r="H76" s="10"/>
       <c r="I76" s="35"/>
       <c r="J76" s="9"/>
@@ -6656,14 +6649,14 @@
       <c r="Z76" s="9"/>
     </row>
     <row r="77" spans="2:26" s="10" customFormat="1" ht="63" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="161" t="s">
+      <c r="B77" s="160" t="s">
         <v>188</v>
       </c>
-      <c r="C77" s="163"/>
-      <c r="D77" s="163"/>
-      <c r="E77" s="163"/>
-      <c r="F77" s="163"/>
-      <c r="G77" s="179"/>
+      <c r="C77" s="161"/>
+      <c r="D77" s="161"/>
+      <c r="E77" s="161"/>
+      <c r="F77" s="161"/>
+      <c r="G77" s="162"/>
     </row>
     <row r="78" spans="2:26" x14ac:dyDescent="0.25">
       <c r="H78" s="10"/>
@@ -6689,50 +6682,9 @@
     <row r="79" spans="2:26" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="63">
-    <mergeCell ref="B77:G77"/>
-    <mergeCell ref="E61:E62"/>
-    <mergeCell ref="G61:G62"/>
-    <mergeCell ref="B65:D67"/>
-    <mergeCell ref="B69:D71"/>
-    <mergeCell ref="B72:D72"/>
-    <mergeCell ref="F69:G71"/>
-    <mergeCell ref="B75:G75"/>
-    <mergeCell ref="B76:G76"/>
-    <mergeCell ref="B52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="E52:E53"/>
-    <mergeCell ref="F52:F53"/>
-    <mergeCell ref="G52:G53"/>
-    <mergeCell ref="B50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="E50:E51"/>
-    <mergeCell ref="F50:F51"/>
-    <mergeCell ref="G50:G51"/>
-    <mergeCell ref="B48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="E48:E49"/>
-    <mergeCell ref="F48:F49"/>
-    <mergeCell ref="G48:G49"/>
-    <mergeCell ref="B46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="G46:G47"/>
-    <mergeCell ref="B44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="E44:E45"/>
-    <mergeCell ref="F44:F45"/>
-    <mergeCell ref="G44:G45"/>
-    <mergeCell ref="E40:E41"/>
-    <mergeCell ref="F40:F41"/>
-    <mergeCell ref="G40:G41"/>
-    <mergeCell ref="B42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="E42:E43"/>
-    <mergeCell ref="F42:F43"/>
-    <mergeCell ref="G42:G43"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="B68:D68"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="G28:G29"/>
     <mergeCell ref="B56:G56"/>
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B5:G5"/>
@@ -6749,12 +6701,53 @@
     <mergeCell ref="D40:D41"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="E40:E41"/>
+    <mergeCell ref="F40:F41"/>
+    <mergeCell ref="G40:G41"/>
+    <mergeCell ref="B42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="E42:E43"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="G42:G43"/>
+    <mergeCell ref="B44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="E44:E45"/>
+    <mergeCell ref="F44:F45"/>
+    <mergeCell ref="G44:G45"/>
+    <mergeCell ref="B46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="G46:G47"/>
+    <mergeCell ref="B48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="E48:E49"/>
+    <mergeCell ref="F48:F49"/>
+    <mergeCell ref="G48:G49"/>
+    <mergeCell ref="B50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="E50:E51"/>
+    <mergeCell ref="F50:F51"/>
+    <mergeCell ref="G50:G51"/>
+    <mergeCell ref="B52:C53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="E52:E53"/>
+    <mergeCell ref="F52:F53"/>
+    <mergeCell ref="G52:G53"/>
+    <mergeCell ref="B77:G77"/>
+    <mergeCell ref="E61:E62"/>
+    <mergeCell ref="G61:G62"/>
+    <mergeCell ref="B65:D67"/>
+    <mergeCell ref="B69:D71"/>
+    <mergeCell ref="B72:D72"/>
+    <mergeCell ref="F69:G71"/>
+    <mergeCell ref="B75:G75"/>
+    <mergeCell ref="B76:G76"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="B68:D68"/>
   </mergeCells>
   <conditionalFormatting sqref="B11:G11 B14:G14 B17:G17 B20:G20 B40:G53 E61 G61 B62:C62 B65:D71 F67 F69:G72 B77:G77">
-    <cfRule type="containsBlanks" dxfId="1" priority="1">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
       <formula>LEN(TRIM(B11))=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6886,124 +6879,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="275" t="s">
+      <c r="A1" s="251" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="275"/>
-      <c r="C1" s="275"/>
-      <c r="D1" s="275"/>
-      <c r="E1" s="275"/>
-      <c r="F1" s="275"/>
-      <c r="G1" s="275"/>
-      <c r="H1" s="275"/>
-      <c r="I1" s="275"/>
-      <c r="J1" s="275"/>
-      <c r="K1" s="275"/>
-      <c r="L1" s="275"/>
-      <c r="M1" s="275"/>
-      <c r="N1" s="275"/>
-      <c r="O1" s="275"/>
-      <c r="P1" s="275"/>
-      <c r="Q1" s="275"/>
-      <c r="R1" s="275"/>
-      <c r="S1" s="275"/>
-      <c r="T1" s="275"/>
-      <c r="U1" s="275" t="s">
+      <c r="B1" s="251"/>
+      <c r="C1" s="251"/>
+      <c r="D1" s="251"/>
+      <c r="E1" s="251"/>
+      <c r="F1" s="251"/>
+      <c r="G1" s="251"/>
+      <c r="H1" s="251"/>
+      <c r="I1" s="251"/>
+      <c r="J1" s="251"/>
+      <c r="K1" s="251"/>
+      <c r="L1" s="251"/>
+      <c r="M1" s="251"/>
+      <c r="N1" s="251"/>
+      <c r="O1" s="251"/>
+      <c r="P1" s="251"/>
+      <c r="Q1" s="251"/>
+      <c r="R1" s="251"/>
+      <c r="S1" s="251"/>
+      <c r="T1" s="251"/>
+      <c r="U1" s="251" t="s">
         <v>159</v>
       </c>
-      <c r="V1" s="275"/>
-      <c r="W1" s="275"/>
-      <c r="X1" s="275"/>
+      <c r="V1" s="251"/>
+      <c r="W1" s="251"/>
+      <c r="X1" s="251"/>
     </row>
     <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="275"/>
-      <c r="B2" s="275"/>
-      <c r="C2" s="275"/>
-      <c r="D2" s="275"/>
-      <c r="E2" s="275"/>
-      <c r="F2" s="275"/>
-      <c r="G2" s="275"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="275"/>
-      <c r="J2" s="275"/>
-      <c r="K2" s="275"/>
-      <c r="L2" s="275"/>
-      <c r="M2" s="275"/>
-      <c r="N2" s="275"/>
-      <c r="O2" s="275"/>
-      <c r="P2" s="275"/>
-      <c r="Q2" s="275"/>
-      <c r="R2" s="275"/>
-      <c r="S2" s="275"/>
-      <c r="T2" s="275"/>
-      <c r="U2" s="255" t="s">
+      <c r="A2" s="251"/>
+      <c r="B2" s="251"/>
+      <c r="C2" s="251"/>
+      <c r="D2" s="251"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="251"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="251"/>
+      <c r="I2" s="251"/>
+      <c r="J2" s="251"/>
+      <c r="K2" s="251"/>
+      <c r="L2" s="251"/>
+      <c r="M2" s="251"/>
+      <c r="N2" s="251"/>
+      <c r="O2" s="251"/>
+      <c r="P2" s="251"/>
+      <c r="Q2" s="251"/>
+      <c r="R2" s="251"/>
+      <c r="S2" s="251"/>
+      <c r="T2" s="251"/>
+      <c r="U2" s="259" t="s">
         <v>160</v>
       </c>
-      <c r="V2" s="255"/>
-      <c r="W2" s="255"/>
-      <c r="X2" s="255"/>
+      <c r="V2" s="259"/>
+      <c r="W2" s="259"/>
+      <c r="X2" s="259"/>
     </row>
     <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="U3" s="282"/>
-      <c r="V3" s="282"/>
-      <c r="W3" s="282"/>
-      <c r="X3" s="282"/>
+      <c r="U3" s="260"/>
+      <c r="V3" s="260"/>
+      <c r="W3" s="260"/>
+      <c r="X3" s="260"/>
     </row>
     <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="279" t="s">
+      <c r="A4" s="256" t="s">
         <v>161</v>
       </c>
-      <c r="B4" s="280"/>
-      <c r="C4" s="280"/>
-      <c r="D4" s="280"/>
-      <c r="E4" s="280"/>
-      <c r="F4" s="280"/>
-      <c r="G4" s="280"/>
-      <c r="H4" s="280"/>
-      <c r="I4" s="280"/>
-      <c r="J4" s="280"/>
-      <c r="K4" s="280"/>
-      <c r="L4" s="280"/>
-      <c r="M4" s="281"/>
-      <c r="N4" s="279" t="s">
+      <c r="B4" s="257"/>
+      <c r="C4" s="257"/>
+      <c r="D4" s="257"/>
+      <c r="E4" s="257"/>
+      <c r="F4" s="257"/>
+      <c r="G4" s="257"/>
+      <c r="H4" s="257"/>
+      <c r="I4" s="257"/>
+      <c r="J4" s="257"/>
+      <c r="K4" s="257"/>
+      <c r="L4" s="257"/>
+      <c r="M4" s="258"/>
+      <c r="N4" s="256" t="s">
         <v>162</v>
       </c>
-      <c r="O4" s="280"/>
-      <c r="P4" s="280"/>
-      <c r="Q4" s="280"/>
-      <c r="R4" s="280"/>
-      <c r="S4" s="280"/>
-      <c r="T4" s="280"/>
-      <c r="U4" s="280"/>
-      <c r="V4" s="280"/>
-      <c r="W4" s="280"/>
-      <c r="X4" s="281"/>
+      <c r="O4" s="257"/>
+      <c r="P4" s="257"/>
+      <c r="Q4" s="257"/>
+      <c r="R4" s="257"/>
+      <c r="S4" s="257"/>
+      <c r="T4" s="257"/>
+      <c r="U4" s="257"/>
+      <c r="V4" s="257"/>
+      <c r="W4" s="257"/>
+      <c r="X4" s="258"/>
     </row>
     <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="276"/>
-      <c r="B5" s="277"/>
-      <c r="C5" s="277"/>
-      <c r="D5" s="277"/>
-      <c r="E5" s="277"/>
-      <c r="F5" s="277"/>
-      <c r="G5" s="277"/>
-      <c r="H5" s="277"/>
-      <c r="I5" s="277"/>
-      <c r="J5" s="277"/>
-      <c r="K5" s="277"/>
-      <c r="L5" s="277"/>
-      <c r="M5" s="278"/>
-      <c r="N5" s="276"/>
-      <c r="O5" s="277"/>
-      <c r="P5" s="277"/>
-      <c r="Q5" s="277"/>
-      <c r="R5" s="277"/>
-      <c r="S5" s="277"/>
-      <c r="T5" s="277"/>
-      <c r="U5" s="277"/>
-      <c r="V5" s="277"/>
-      <c r="W5" s="277"/>
-      <c r="X5" s="278"/>
+      <c r="A5" s="253"/>
+      <c r="B5" s="254"/>
+      <c r="C5" s="254"/>
+      <c r="D5" s="254"/>
+      <c r="E5" s="254"/>
+      <c r="F5" s="254"/>
+      <c r="G5" s="254"/>
+      <c r="H5" s="254"/>
+      <c r="I5" s="254"/>
+      <c r="J5" s="254"/>
+      <c r="K5" s="254"/>
+      <c r="L5" s="254"/>
+      <c r="M5" s="255"/>
+      <c r="N5" s="253"/>
+      <c r="O5" s="254"/>
+      <c r="P5" s="254"/>
+      <c r="Q5" s="254"/>
+      <c r="R5" s="254"/>
+      <c r="S5" s="254"/>
+      <c r="T5" s="254"/>
+      <c r="U5" s="254"/>
+      <c r="V5" s="254"/>
+      <c r="W5" s="254"/>
+      <c r="X5" s="255"/>
     </row>
     <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
@@ -7032,66 +7025,66 @@
       <c r="X6" s="3"/>
     </row>
     <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="253" t="s">
+      <c r="A7" s="252" t="s">
         <v>163</v>
       </c>
-      <c r="B7" s="253"/>
-      <c r="C7" s="253"/>
-      <c r="D7" s="253"/>
-      <c r="E7" s="253"/>
-      <c r="F7" s="253"/>
-      <c r="G7" s="253"/>
-      <c r="H7" s="253"/>
-      <c r="I7" s="253"/>
-      <c r="J7" s="253" t="s">
+      <c r="B7" s="252"/>
+      <c r="C7" s="252"/>
+      <c r="D7" s="252"/>
+      <c r="E7" s="252"/>
+      <c r="F7" s="252"/>
+      <c r="G7" s="252"/>
+      <c r="H7" s="252"/>
+      <c r="I7" s="252"/>
+      <c r="J7" s="252" t="s">
         <v>32</v>
       </c>
-      <c r="K7" s="253"/>
-      <c r="L7" s="253"/>
-      <c r="M7" s="253"/>
-      <c r="N7" s="253"/>
-      <c r="O7" s="253"/>
-      <c r="P7" s="253" t="s">
+      <c r="K7" s="252"/>
+      <c r="L7" s="252"/>
+      <c r="M7" s="252"/>
+      <c r="N7" s="252"/>
+      <c r="O7" s="252"/>
+      <c r="P7" s="252" t="s">
         <v>58</v>
       </c>
-      <c r="Q7" s="253"/>
-      <c r="R7" s="253"/>
-      <c r="S7" s="253"/>
-      <c r="T7" s="253"/>
-      <c r="U7" s="253"/>
-      <c r="V7" s="253"/>
-      <c r="W7" s="253"/>
-      <c r="X7" s="253"/>
+      <c r="Q7" s="252"/>
+      <c r="R7" s="252"/>
+      <c r="S7" s="252"/>
+      <c r="T7" s="252"/>
+      <c r="U7" s="252"/>
+      <c r="V7" s="252"/>
+      <c r="W7" s="252"/>
+      <c r="X7" s="252"/>
     </row>
     <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="260"/>
-      <c r="B8" s="260"/>
-      <c r="C8" s="260"/>
-      <c r="D8" s="260"/>
-      <c r="E8" s="260"/>
-      <c r="F8" s="260"/>
-      <c r="G8" s="260"/>
-      <c r="H8" s="260"/>
-      <c r="I8" s="260"/>
-      <c r="J8" s="261" t="s">
+      <c r="A8" s="261"/>
+      <c r="B8" s="261"/>
+      <c r="C8" s="261"/>
+      <c r="D8" s="261"/>
+      <c r="E8" s="261"/>
+      <c r="F8" s="261"/>
+      <c r="G8" s="261"/>
+      <c r="H8" s="261"/>
+      <c r="I8" s="261"/>
+      <c r="J8" s="262" t="s">
         <v>164</v>
       </c>
-      <c r="K8" s="262"/>
-      <c r="L8" s="262"/>
-      <c r="M8" s="262"/>
-      <c r="N8" s="262"/>
-      <c r="O8" s="263"/>
-      <c r="P8" s="261" t="s">
+      <c r="K8" s="263"/>
+      <c r="L8" s="263"/>
+      <c r="M8" s="263"/>
+      <c r="N8" s="263"/>
+      <c r="O8" s="264"/>
+      <c r="P8" s="262" t="s">
         <v>165</v>
       </c>
-      <c r="Q8" s="262"/>
-      <c r="R8" s="262"/>
-      <c r="S8" s="262"/>
-      <c r="T8" s="262"/>
-      <c r="U8" s="262"/>
-      <c r="V8" s="262"/>
-      <c r="W8" s="262"/>
-      <c r="X8" s="263"/>
+      <c r="Q8" s="263"/>
+      <c r="R8" s="263"/>
+      <c r="S8" s="263"/>
+      <c r="T8" s="263"/>
+      <c r="U8" s="263"/>
+      <c r="V8" s="263"/>
+      <c r="W8" s="263"/>
+      <c r="X8" s="264"/>
     </row>
     <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
@@ -7120,66 +7113,66 @@
       <c r="X9" s="3"/>
     </row>
     <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="273" t="s">
+      <c r="A10" s="265" t="s">
         <v>166</v>
       </c>
-      <c r="B10" s="273"/>
-      <c r="C10" s="273"/>
-      <c r="D10" s="273"/>
-      <c r="E10" s="273"/>
-      <c r="F10" s="273"/>
-      <c r="G10" s="273"/>
-      <c r="H10" s="273"/>
-      <c r="I10" s="273"/>
-      <c r="J10" s="273"/>
-      <c r="K10" s="273"/>
-      <c r="L10" s="273"/>
-      <c r="M10" s="273"/>
-      <c r="N10" s="273"/>
-      <c r="O10" s="273"/>
-      <c r="P10" s="273"/>
-      <c r="Q10" s="273"/>
-      <c r="R10" s="273"/>
-      <c r="S10" s="273"/>
-      <c r="T10" s="273"/>
-      <c r="U10" s="273"/>
-      <c r="V10" s="273"/>
-      <c r="W10" s="273"/>
-      <c r="X10" s="273"/>
+      <c r="B10" s="265"/>
+      <c r="C10" s="265"/>
+      <c r="D10" s="265"/>
+      <c r="E10" s="265"/>
+      <c r="F10" s="265"/>
+      <c r="G10" s="265"/>
+      <c r="H10" s="265"/>
+      <c r="I10" s="265"/>
+      <c r="J10" s="265"/>
+      <c r="K10" s="265"/>
+      <c r="L10" s="265"/>
+      <c r="M10" s="265"/>
+      <c r="N10" s="265"/>
+      <c r="O10" s="265"/>
+      <c r="P10" s="265"/>
+      <c r="Q10" s="265"/>
+      <c r="R10" s="265"/>
+      <c r="S10" s="265"/>
+      <c r="T10" s="265"/>
+      <c r="U10" s="265"/>
+      <c r="V10" s="265"/>
+      <c r="W10" s="265"/>
+      <c r="X10" s="265"/>
     </row>
     <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="274" t="s">
+      <c r="A11" s="266" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="274"/>
-      <c r="C11" s="274"/>
-      <c r="D11" s="274"/>
-      <c r="E11" s="274"/>
-      <c r="F11" s="274"/>
-      <c r="G11" s="274" t="s">
+      <c r="B11" s="266"/>
+      <c r="C11" s="266"/>
+      <c r="D11" s="266"/>
+      <c r="E11" s="266"/>
+      <c r="F11" s="266"/>
+      <c r="G11" s="266" t="s">
         <v>167</v>
       </c>
-      <c r="H11" s="274"/>
-      <c r="I11" s="274"/>
-      <c r="J11" s="274"/>
-      <c r="K11" s="274"/>
-      <c r="L11" s="274"/>
-      <c r="M11" s="274" t="s">
+      <c r="H11" s="266"/>
+      <c r="I11" s="266"/>
+      <c r="J11" s="266"/>
+      <c r="K11" s="266"/>
+      <c r="L11" s="266"/>
+      <c r="M11" s="266" t="s">
         <v>168</v>
       </c>
-      <c r="N11" s="274"/>
-      <c r="O11" s="274"/>
-      <c r="P11" s="274"/>
-      <c r="Q11" s="274"/>
-      <c r="R11" s="274"/>
-      <c r="S11" s="274" t="s">
+      <c r="N11" s="266"/>
+      <c r="O11" s="266"/>
+      <c r="P11" s="266"/>
+      <c r="Q11" s="266"/>
+      <c r="R11" s="266"/>
+      <c r="S11" s="266" t="s">
         <v>169</v>
       </c>
-      <c r="T11" s="274"/>
-      <c r="U11" s="274"/>
-      <c r="V11" s="274"/>
-      <c r="W11" s="274"/>
-      <c r="X11" s="274"/>
+      <c r="T11" s="266"/>
+      <c r="U11" s="266"/>
+      <c r="V11" s="266"/>
+      <c r="W11" s="266"/>
+      <c r="X11" s="266"/>
     </row>
     <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
@@ -7208,66 +7201,66 @@
       <c r="X12" s="3"/>
     </row>
     <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="253" t="s">
+      <c r="A13" s="252" t="s">
         <v>170</v>
       </c>
-      <c r="B13" s="253"/>
-      <c r="C13" s="253"/>
-      <c r="D13" s="253"/>
-      <c r="E13" s="253"/>
-      <c r="F13" s="253"/>
-      <c r="G13" s="253"/>
-      <c r="H13" s="253"/>
-      <c r="I13" s="253"/>
-      <c r="J13" s="253" t="s">
+      <c r="B13" s="252"/>
+      <c r="C13" s="252"/>
+      <c r="D13" s="252"/>
+      <c r="E13" s="252"/>
+      <c r="F13" s="252"/>
+      <c r="G13" s="252"/>
+      <c r="H13" s="252"/>
+      <c r="I13" s="252"/>
+      <c r="J13" s="252" t="s">
         <v>32</v>
       </c>
-      <c r="K13" s="253"/>
-      <c r="L13" s="253"/>
-      <c r="M13" s="253"/>
-      <c r="N13" s="253"/>
-      <c r="O13" s="253"/>
-      <c r="P13" s="253" t="s">
+      <c r="K13" s="252"/>
+      <c r="L13" s="252"/>
+      <c r="M13" s="252"/>
+      <c r="N13" s="252"/>
+      <c r="O13" s="252"/>
+      <c r="P13" s="252" t="s">
         <v>58</v>
       </c>
-      <c r="Q13" s="253"/>
-      <c r="R13" s="253"/>
-      <c r="S13" s="253"/>
-      <c r="T13" s="253"/>
-      <c r="U13" s="253"/>
-      <c r="V13" s="253"/>
-      <c r="W13" s="253"/>
-      <c r="X13" s="253"/>
+      <c r="Q13" s="252"/>
+      <c r="R13" s="252"/>
+      <c r="S13" s="252"/>
+      <c r="T13" s="252"/>
+      <c r="U13" s="252"/>
+      <c r="V13" s="252"/>
+      <c r="W13" s="252"/>
+      <c r="X13" s="252"/>
     </row>
     <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="260"/>
-      <c r="B14" s="260"/>
-      <c r="C14" s="260"/>
-      <c r="D14" s="260"/>
-      <c r="E14" s="260"/>
-      <c r="F14" s="260"/>
-      <c r="G14" s="260"/>
-      <c r="H14" s="260"/>
-      <c r="I14" s="260"/>
-      <c r="J14" s="261" t="s">
+      <c r="A14" s="261"/>
+      <c r="B14" s="261"/>
+      <c r="C14" s="261"/>
+      <c r="D14" s="261"/>
+      <c r="E14" s="261"/>
+      <c r="F14" s="261"/>
+      <c r="G14" s="261"/>
+      <c r="H14" s="261"/>
+      <c r="I14" s="261"/>
+      <c r="J14" s="262" t="s">
         <v>171</v>
       </c>
-      <c r="K14" s="262"/>
-      <c r="L14" s="262"/>
-      <c r="M14" s="262"/>
-      <c r="N14" s="262"/>
-      <c r="O14" s="263"/>
-      <c r="P14" s="261" t="s">
+      <c r="K14" s="263"/>
+      <c r="L14" s="263"/>
+      <c r="M14" s="263"/>
+      <c r="N14" s="263"/>
+      <c r="O14" s="264"/>
+      <c r="P14" s="262" t="s">
         <v>172</v>
       </c>
-      <c r="Q14" s="262"/>
-      <c r="R14" s="262"/>
-      <c r="S14" s="262"/>
-      <c r="T14" s="262"/>
-      <c r="U14" s="262"/>
-      <c r="V14" s="262"/>
-      <c r="W14" s="262"/>
-      <c r="X14" s="263"/>
+      <c r="Q14" s="263"/>
+      <c r="R14" s="263"/>
+      <c r="S14" s="263"/>
+      <c r="T14" s="263"/>
+      <c r="U14" s="263"/>
+      <c r="V14" s="263"/>
+      <c r="W14" s="263"/>
+      <c r="X14" s="264"/>
     </row>
     <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
@@ -7296,184 +7289,172 @@
       <c r="X15" s="3"/>
     </row>
     <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="264" t="s">
+      <c r="A16" s="272" t="s">
         <v>173</v>
       </c>
-      <c r="B16" s="264"/>
-      <c r="C16" s="264"/>
-      <c r="D16" s="264"/>
-      <c r="E16" s="264"/>
-      <c r="F16" s="264"/>
-      <c r="G16" s="264"/>
-      <c r="H16" s="264"/>
-      <c r="I16" s="264"/>
-      <c r="J16" s="265" t="s">
+      <c r="B16" s="272"/>
+      <c r="C16" s="272"/>
+      <c r="D16" s="272"/>
+      <c r="E16" s="272"/>
+      <c r="F16" s="272"/>
+      <c r="G16" s="272"/>
+      <c r="H16" s="272"/>
+      <c r="I16" s="272"/>
+      <c r="J16" s="273" t="s">
         <v>174</v>
       </c>
-      <c r="K16" s="265"/>
-      <c r="L16" s="265"/>
-      <c r="M16" s="265"/>
-      <c r="N16" s="264" t="s">
+      <c r="K16" s="273"/>
+      <c r="L16" s="273"/>
+      <c r="M16" s="273"/>
+      <c r="N16" s="272" t="s">
         <v>175</v>
       </c>
-      <c r="O16" s="264"/>
-      <c r="P16" s="264"/>
-      <c r="Q16" s="264"/>
-      <c r="R16" s="264"/>
-      <c r="S16" s="264"/>
-      <c r="T16" s="266" t="s">
+      <c r="O16" s="272"/>
+      <c r="P16" s="272"/>
+      <c r="Q16" s="272"/>
+      <c r="R16" s="272"/>
+      <c r="S16" s="272"/>
+      <c r="T16" s="274" t="s">
         <v>176</v>
       </c>
-      <c r="U16" s="266"/>
-      <c r="V16" s="266"/>
-      <c r="W16" s="266"/>
-      <c r="X16" s="266"/>
+      <c r="U16" s="274"/>
+      <c r="V16" s="274"/>
+      <c r="W16" s="274"/>
+      <c r="X16" s="274"/>
     </row>
     <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="254" t="s">
+      <c r="A17" s="267" t="s">
         <v>177</v>
       </c>
-      <c r="B17" s="255"/>
-      <c r="C17" s="255"/>
-      <c r="D17" s="255"/>
-      <c r="E17" s="255"/>
-      <c r="F17" s="255"/>
-      <c r="G17" s="255"/>
-      <c r="H17" s="255"/>
-      <c r="I17" s="256"/>
-      <c r="J17" s="267" t="s">
+      <c r="B17" s="259"/>
+      <c r="C17" s="259"/>
+      <c r="D17" s="259"/>
+      <c r="E17" s="259"/>
+      <c r="F17" s="259"/>
+      <c r="G17" s="259"/>
+      <c r="H17" s="259"/>
+      <c r="I17" s="268"/>
+      <c r="J17" s="275" t="s">
         <v>178</v>
       </c>
-      <c r="K17" s="268"/>
-      <c r="L17" s="268"/>
-      <c r="M17" s="269"/>
-      <c r="N17" s="254" t="s">
+      <c r="K17" s="276"/>
+      <c r="L17" s="276"/>
+      <c r="M17" s="277"/>
+      <c r="N17" s="267" t="s">
         <v>179</v>
       </c>
-      <c r="O17" s="255"/>
-      <c r="P17" s="255"/>
-      <c r="Q17" s="255"/>
-      <c r="R17" s="255"/>
-      <c r="S17" s="256"/>
-      <c r="T17" s="254" t="s">
+      <c r="O17" s="259"/>
+      <c r="P17" s="259"/>
+      <c r="Q17" s="259"/>
+      <c r="R17" s="259"/>
+      <c r="S17" s="268"/>
+      <c r="T17" s="267" t="s">
         <v>180</v>
       </c>
-      <c r="U17" s="255"/>
-      <c r="V17" s="255"/>
-      <c r="W17" s="255"/>
-      <c r="X17" s="256"/>
+      <c r="U17" s="259"/>
+      <c r="V17" s="259"/>
+      <c r="W17" s="259"/>
+      <c r="X17" s="268"/>
     </row>
     <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="257"/>
-      <c r="B18" s="258"/>
-      <c r="C18" s="258"/>
-      <c r="D18" s="258"/>
-      <c r="E18" s="258"/>
-      <c r="F18" s="258"/>
-      <c r="G18" s="258"/>
-      <c r="H18" s="258"/>
-      <c r="I18" s="259"/>
-      <c r="J18" s="270"/>
-      <c r="K18" s="271"/>
-      <c r="L18" s="271"/>
-      <c r="M18" s="272"/>
-      <c r="N18" s="257"/>
-      <c r="O18" s="258"/>
-      <c r="P18" s="258"/>
-      <c r="Q18" s="258"/>
-      <c r="R18" s="258"/>
-      <c r="S18" s="259"/>
-      <c r="T18" s="257"/>
-      <c r="U18" s="258"/>
-      <c r="V18" s="258"/>
-      <c r="W18" s="258"/>
-      <c r="X18" s="259"/>
+      <c r="A18" s="269"/>
+      <c r="B18" s="270"/>
+      <c r="C18" s="270"/>
+      <c r="D18" s="270"/>
+      <c r="E18" s="270"/>
+      <c r="F18" s="270"/>
+      <c r="G18" s="270"/>
+      <c r="H18" s="270"/>
+      <c r="I18" s="271"/>
+      <c r="J18" s="278"/>
+      <c r="K18" s="279"/>
+      <c r="L18" s="279"/>
+      <c r="M18" s="280"/>
+      <c r="N18" s="269"/>
+      <c r="O18" s="270"/>
+      <c r="P18" s="270"/>
+      <c r="Q18" s="270"/>
+      <c r="R18" s="270"/>
+      <c r="S18" s="271"/>
+      <c r="T18" s="269"/>
+      <c r="U18" s="270"/>
+      <c r="V18" s="270"/>
+      <c r="W18" s="270"/>
+      <c r="X18" s="271"/>
     </row>
     <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A21" s="252" t="s">
+      <c r="A21" s="284" t="s">
         <v>181</v>
       </c>
-      <c r="B21" s="252"/>
-      <c r="C21" s="252"/>
-      <c r="D21" s="252"/>
-      <c r="E21" s="252"/>
-      <c r="F21" s="252"/>
-      <c r="G21" s="252"/>
-      <c r="H21" s="252"/>
+      <c r="B21" s="284"/>
+      <c r="C21" s="284"/>
+      <c r="D21" s="284"/>
+      <c r="E21" s="284"/>
+      <c r="F21" s="284"/>
+      <c r="G21" s="284"/>
+      <c r="H21" s="284"/>
       <c r="I21" s="5"/>
-      <c r="J21" s="252" t="s">
+      <c r="J21" s="284" t="s">
         <v>182</v>
       </c>
-      <c r="K21" s="252"/>
-      <c r="L21" s="252"/>
-      <c r="M21" s="252"/>
-      <c r="N21" s="252"/>
-      <c r="O21" s="252"/>
-      <c r="P21" s="252"/>
+      <c r="K21" s="284"/>
+      <c r="L21" s="284"/>
+      <c r="M21" s="284"/>
+      <c r="N21" s="284"/>
+      <c r="O21" s="284"/>
+      <c r="P21" s="284"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="252" t="s">
+      <c r="R21" s="284" t="s">
         <v>183</v>
       </c>
-      <c r="S21" s="252"/>
-      <c r="T21" s="252"/>
-      <c r="U21" s="252"/>
-      <c r="V21" s="252"/>
-      <c r="W21" s="252"/>
-      <c r="X21" s="252"/>
+      <c r="S21" s="284"/>
+      <c r="T21" s="284"/>
+      <c r="U21" s="284"/>
+      <c r="V21" s="284"/>
+      <c r="W21" s="284"/>
+      <c r="X21" s="284"/>
     </row>
     <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P23" s="249" t="s">
+      <c r="P23" s="281" t="s">
         <v>184</v>
       </c>
-      <c r="Q23" s="249"/>
-      <c r="R23" s="249"/>
-      <c r="S23" s="249"/>
-      <c r="T23" s="249"/>
-      <c r="U23" s="250" t="s">
+      <c r="Q23" s="281"/>
+      <c r="R23" s="281"/>
+      <c r="S23" s="281"/>
+      <c r="T23" s="281"/>
+      <c r="U23" s="282" t="s">
         <v>185</v>
       </c>
-      <c r="V23" s="250"/>
-      <c r="W23" s="250"/>
-      <c r="X23" s="250"/>
+      <c r="V23" s="282"/>
+      <c r="W23" s="282"/>
+      <c r="X23" s="282"/>
     </row>
     <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P24" s="249" t="s">
+      <c r="P24" s="281" t="s">
         <v>186</v>
       </c>
-      <c r="Q24" s="249"/>
-      <c r="R24" s="249"/>
-      <c r="S24" s="249"/>
-      <c r="T24" s="249"/>
-      <c r="U24" s="251" t="s">
+      <c r="Q24" s="281"/>
+      <c r="R24" s="281"/>
+      <c r="S24" s="281"/>
+      <c r="T24" s="281"/>
+      <c r="U24" s="283" t="s">
         <v>187</v>
       </c>
-      <c r="V24" s="251"/>
-      <c r="W24" s="251"/>
-      <c r="X24" s="251"/>
+      <c r="V24" s="283"/>
+      <c r="W24" s="283"/>
+      <c r="X24" s="283"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="J7:O7"/>
-    <mergeCell ref="P7:X7"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="N4:X4"/>
-    <mergeCell ref="N5:X5"/>
-    <mergeCell ref="U2:X3"/>
-    <mergeCell ref="A8:I8"/>
-    <mergeCell ref="J8:O8"/>
-    <mergeCell ref="P8:X8"/>
-    <mergeCell ref="A10:X10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="G11:L11"/>
-    <mergeCell ref="M11:R11"/>
-    <mergeCell ref="S11:X11"/>
+    <mergeCell ref="P23:T23"/>
+    <mergeCell ref="U23:X23"/>
+    <mergeCell ref="P24:T24"/>
+    <mergeCell ref="U24:X24"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="J21:P21"/>
+    <mergeCell ref="R21:X21"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="J13:O13"/>
     <mergeCell ref="P13:X13"/>
@@ -7488,13 +7469,25 @@
     <mergeCell ref="T16:X16"/>
     <mergeCell ref="A17:I18"/>
     <mergeCell ref="J17:M18"/>
-    <mergeCell ref="P23:T23"/>
-    <mergeCell ref="U23:X23"/>
-    <mergeCell ref="P24:T24"/>
-    <mergeCell ref="U24:X24"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="J21:P21"/>
-    <mergeCell ref="R21:X21"/>
+    <mergeCell ref="A8:I8"/>
+    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="P8:X8"/>
+    <mergeCell ref="A10:X10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="G11:L11"/>
+    <mergeCell ref="M11:R11"/>
+    <mergeCell ref="S11:X11"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="A2:T2"/>
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="J7:O7"/>
+    <mergeCell ref="P7:X7"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A4:M4"/>
+    <mergeCell ref="N4:X4"/>
+    <mergeCell ref="N5:X5"/>
+    <mergeCell ref="U2:X3"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="95" orientation="landscape" horizontalDpi="4294967294" verticalDpi="200" r:id="rId1"/>
@@ -7512,6 +7505,21 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010080239B14884FBB46AB47CE62E6B5D997" ma:contentTypeVersion="23" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="7588953d79b37feb9934caf9b24b5887">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="edbb1c21-1b45-407e-8894-c97732534993" xmlns:ns3="41dd0a9e-964d-48c8-9389-7445c2a187f7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e8a576e1ff98af8803e81906898dd43d" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -7801,21 +7809,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="41dd0a9e-964d-48c8-9389-7445c2a187f7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="edbb1c21-1b45-407e-8894-c97732534993">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <FechayHora xmlns="edbb1c21-1b45-407e-8894-c97732534993" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CCE7917-804F-4951-9FEA-F53AEA82B8BE}">
   <ds:schemaRefs>
@@ -7825,6 +7818,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBE5A30C-34BC-4387-870E-CFF8B53C216A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
+    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B283548F-AD1F-4BAB-8C10-49DF5F0AEBA9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7842,16 +7847,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBE5A30C-34BC-4387-870E-CFF8B53C216A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="41dd0a9e-964d-48c8-9389-7445c2a187f7"/>
-    <ds:schemaRef ds:uri="edbb1c21-1b45-407e-8894-c97732534993"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>